<commit_message>
Enforce: Align 100% of student roster, room, classNo, gender, and spelling to official school registry XLS
</commit_message>
<xml_diff>
--- a/เอกสารและรายชื่อคณะสีแสด_ปี69/แยกฝ่าย/ดรัมเมเยอร์/รายชื่อดรัมเมเยอร์_คณะสีแสด_ปี69.xlsx
+++ b/เอกสารและรายชื่อคณะสีแสด_ปี69/แยกฝ่าย/ดรัมเมเยอร์/รายชื่อดรัมเมเยอร์_คณะสีแสด_ปี69.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="34">
   <si>
     <t>🥁 รายชื่อสมาชิกฝ่ายดรัมเมเยอร์ — คณะสีแสด (สีบุษราคัม) ปี 2569</t>
   </si>
@@ -40,9 +40,6 @@
     <t>เบอร์โทรศัพท์</t>
   </si>
   <si>
-    <t>ม.4/13</t>
-  </si>
-  <si>
     <t>33130</t>
   </si>
   <si>
@@ -55,9 +52,6 @@
     <t>098-817-0691</t>
   </si>
   <si>
-    <t>ม.3/5</t>
-  </si>
-  <si>
     <t>33803</t>
   </si>
   <si>
@@ -76,9 +70,6 @@
     <t>096-359-4382</t>
   </si>
   <si>
-    <t>ม.3/6</t>
-  </si>
-  <si>
     <t>33845</t>
   </si>
   <si>
@@ -88,9 +79,6 @@
     <t>080-800-6634</t>
   </si>
   <si>
-    <t>ม.3/1</t>
-  </si>
-  <si>
     <t>33641</t>
   </si>
   <si>
@@ -100,9 +88,6 @@
     <t>099-616-9767</t>
   </si>
   <si>
-    <t>ม.5/4</t>
-  </si>
-  <si>
     <t>32631</t>
   </si>
   <si>
@@ -119,9 +104,6 @@
   </si>
   <si>
     <t>061-553-0691</t>
-  </si>
-  <si>
-    <t>ม.5/6</t>
   </si>
   <si>
     <t>32653</t>
@@ -661,184 +643,168 @@
       <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="B4" s="4"/>
       <c r="C4" s="4">
         <v>17</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
         <v>2</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>14</v>
-      </c>
+      <c r="B5" s="6"/>
       <c r="C5" s="6">
         <v>28</v>
       </c>
       <c r="D5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>15</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="B6" s="4"/>
       <c r="C6" s="4">
         <v>23</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6">
         <v>4</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>21</v>
-      </c>
+      <c r="B7" s="6"/>
       <c r="C7" s="6">
         <v>30</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="B8" s="4"/>
       <c r="C8" s="4">
         <v>27</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>6</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="B9" s="6"/>
       <c r="C9" s="6">
         <v>30</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>7</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>29</v>
-      </c>
+      <c r="B10" s="4"/>
       <c r="C10" s="4">
         <v>23</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="6">
         <v>8</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>36</v>
-      </c>
+      <c r="B11" s="6"/>
       <c r="C11" s="6">
         <v>25</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>